<commit_message>
Updated WDC to remove one time cash gain
</commit_message>
<xml_diff>
--- a/STX.xlsx
+++ b/STX.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F40004B-F03F-E745-9B4A-7BA75D0CF613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1020F86A-FA10-8942-B689-E9A1C9EDD4F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
@@ -137,7 +137,7 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="2">
+  <futureMetadata name="XLRICHVALUE" count="5">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -148,7 +148,28 @@
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="8"/>
         </ext>
       </extLst>
     </bk>
@@ -158,12 +179,21 @@
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="2">
+  <valueMetadata count="5">
     <bk>
       <rc t="2" v="0"/>
     </bk>
     <bk>
       <rc t="2" v="1"/>
+    </bk>
+    <bk>
+      <rc t="2" v="2"/>
+    </bk>
+    <bk>
+      <rc t="2" v="3"/>
+    </bk>
+    <bk>
+      <rc t="2" v="4"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -2452,6 +2482,12 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2459,12 +2495,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2485,14 +2515,14 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -12661,7 +12691,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="6">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="9">
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a23rjc&amp;q=XNAS%3aSTX&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
@@ -12680,11 +12710,9 @@
     <v>Powered by Refinitiv</v>
     <v>1145</v>
     <v>209</v>
-    <v>2.1537000000000002</v>
-    <v>21.8</v>
-    <v>3.4114999999999999E-2</v>
-    <v>0.09</v>
-    <v>1.362E-4</v>
+    <v>2.1414</v>
+    <v>15.955</v>
+    <v>2.4145E-2</v>
     <v>USD</v>
     <v>Seagate Technology Holdings plc provides mass-data storage infrastructure solution. The Company’s principal products are hard disk drives, commonly referred to as disk drives, hard drives (HDDs). In addition to HDDs, the Company produces a range of data storage products, including solid state drives (SSDs), solid state hybrid drives, storage subsystems, as well as a scalable edge-to-cloud mass data platform. Its HDD products are designed for mass capacity storage and legacy markets. Mass capacity storage involves use cases, such as hyperscale data centers and public clouds, as well as emerging use cases. The Company’s HDD and SSD product portfolio includes Serial Advanced Technology Attachment, Serial Attached SCSI and Non-Volatile Memory Express based designs to support a variety of mass capacity and legacy applications. Its systems portfolio includes storage subsystems for enterprises, cloud service providers, scale-out storage servers and original equipment manufacturers.</v>
     <v>30000</v>
@@ -12692,35 +12720,49 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>121 Woodlands Avenue 5, 739009 SG</v>
-    <v>675.70659999999998</v>
+    <v>679.8</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46314.919582036717</v>
+    <v>46315.694664108596</v>
     <v>0</v>
-    <v>654.52</v>
-    <v>151352517129</v>
+    <v>642.41999999999996</v>
+    <v>155006864688</v>
     <v>SEAGATE TECHNOLOGY HOLDINGS PUBLIC LIMITED COMPANY</v>
     <v>SEAGATE TECHNOLOGY HOLDINGS PUBLIC LIMITED COMPANY</v>
-    <v>665</v>
-    <v>45.9589</v>
-    <v>639.01</v>
+    <v>657.17</v>
+    <v>48.674500000000002</v>
     <v>660.81</v>
-    <v>660.9</v>
+    <v>676.76499999999999</v>
     <v>229040900</v>
     <v>STX</v>
     <v>SEAGATE TECHNOLOGY HOLDINGS PUBLIC LIMITED COMPANY (XNAS:STX)</v>
-    <v>4127674</v>
-    <v>4841848</v>
+    <v>2232223</v>
+    <v>4841084</v>
     <v>2017</v>
   </rv>
   <rv s="2">
     <v>1</v>
   </rv>
+  <rv s="3">
+    <v>12</v>
+    <v>Price (Extended hours)</v>
+    <v>0</v>
+  </rv>
+  <rv s="3">
+    <v>12</v>
+    <v>Change (extended hours)</v>
+    <v>0</v>
+  </rv>
+  <rv s="3">
+    <v>12</v>
+    <v>Change % (extended hours)</v>
+    <v>0</v>
+  </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a33knm&amp;q=10+Y+TSY+YLD+NDX&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="3">
+  <rv s="4">
     <v>5</v>
     <v>10 Y TSY YLD NDX</v>
     <v>6</v>
@@ -12734,28 +12776,28 @@
     <v>Powered by Refinitiv</v>
     <v>53.64</v>
     <v>39.47</v>
-    <v>0.09</v>
-    <v>1.769E-3</v>
+    <v>0.38</v>
+    <v>7.4539999999999997E-3</v>
     <v>US</v>
-    <v>51.33</v>
+    <v>51.5</v>
     <v>Index</v>
-    <v>3</v>
-    <v>50.67</v>
+    <v>6</v>
+    <v>50.9</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>51.14</v>
-    <v>50.89</v>
+    <v>50.9</v>
     <v>50.98</v>
+    <v>51.36</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
   <rv s="2">
-    <v>4</v>
+    <v>7</v>
   </rv>
 </rvData>
 </file>
 
 <file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="5">
   <s t="_hyperlink">
     <k n="Address" t="s"/>
     <k n="Text" t="s"/>
@@ -12777,8 +12819,6 @@
     <k n="Beta"/>
     <k n="Change"/>
     <k n="Change (%)"/>
-    <k n="Change (Extended hours)"/>
-    <k n="Change % (Extended hours)"/>
     <k n="Currency" t="s"/>
     <k n="Description" t="s"/>
     <k n="Employees"/>
@@ -12799,7 +12839,6 @@
     <k n="P/E"/>
     <k n="Previous close"/>
     <k n="Price"/>
-    <k n="Price (Extended hours)"/>
     <k n="Shares outstanding"/>
     <k n="Ticker symbol" t="s"/>
     <k n="UniqueName" t="s"/>
@@ -12809,6 +12848,11 @@
   </s>
   <s t="_linkedentity">
     <k n="%cvi" t="r"/>
+  </s>
+  <s t="_error">
+    <k n="errorType" t="i"/>
+    <k n="field" t="s"/>
+    <k n="subType" t="i"/>
   </s>
   <s t="_linkedentitycore">
     <k n="_Display" t="spb"/>
@@ -12844,7 +12888,7 @@
 <file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
 <supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
   <spbArrays count="2">
-    <a count="45">
+    <a count="42">
       <v t="s">%EntityServiceId</v>
       <v t="s">_Format</v>
       <v t="s">%IsRefreshable</v>
@@ -12855,16 +12899,13 @@
       <v t="s">Name</v>
       <v t="s">_SubLabel</v>
       <v t="s">Price</v>
-      <v t="s">Price (Extended hours)</v>
       <v t="s">Exchange</v>
       <v t="s">Official name</v>
       <v t="s">Last trade time</v>
       <v t="s">Ticker symbol</v>
       <v t="s">Exchange abbreviation</v>
       <v t="s">Change</v>
-      <v t="s">Change (Extended hours)</v>
       <v t="s">Change (%)</v>
-      <v t="s">Change % (Extended hours)</v>
       <v t="s">Currency</v>
       <v t="s">Previous close</v>
       <v t="s">Open</v>
@@ -12958,19 +12999,13 @@
       <v>8</v>
       <v>9</v>
       <v>4</v>
-      <v>1</v>
-      <v>1</v>
-      <v>5</v>
     </spb>
     <spb s="4">
-      <v>at close</v>
+      <v>Real-Time Nasdaq Last Sale</v>
       <v>from previous close</v>
       <v>from previous close</v>
       <v>Source: Nasdaq Last Sale</v>
       <v>GMT</v>
-      <v>Real-Time Nasdaq Last Sale</v>
-      <v>from close</v>
-      <v>from close</v>
     </spb>
     <spb s="0">
       <v>1</v>
@@ -13042,9 +13077,6 @@
     <k n="Year incorporated" t="i"/>
     <k n="`%EntityServiceId" t="i"/>
     <k n="Shares outstanding" t="i"/>
-    <k n="Price (Extended hours)" t="i"/>
-    <k n="Change (Extended hours)" t="i"/>
-    <k n="Change % (Extended hours)" t="i"/>
   </s>
   <s>
     <k n="Price" t="s"/>
@@ -13052,9 +13084,6 @@
     <k n="Change (%)" t="s"/>
     <k n="ExchangeID" t="s"/>
     <k n="Last trade time" t="s"/>
-    <k n="Price (Extended hours)" t="s"/>
-    <k n="Change (Extended hours)" t="s"/>
-    <k n="Change % (Extended hours)" t="s"/>
   </s>
   <s>
     <k n="UniqueName" t="spb"/>
@@ -13577,7 +13606,7 @@
       </c>
       <c r="F3" s="183">
         <f ca="1">Statement!AC151</f>
-        <v>156611.97</v>
+        <v>160393.30499999999</v>
       </c>
       <c r="H3" s="181" t="str">
         <f>'AVG target price'!B5</f>
@@ -13585,7 +13614,7 @@
       </c>
       <c r="I3" s="207">
         <f ca="1">'AVG target price'!C5</f>
-        <v>133.36063643452346</v>
+        <v>133.47386617275473</v>
       </c>
       <c r="K3" s="244" t="s">
         <v>435</v>
@@ -13604,7 +13633,7 @@
       </c>
       <c r="F4" s="184">
         <f ca="1">Statement!AC152</f>
-        <v>158472.97</v>
+        <v>162254.30499999999</v>
       </c>
       <c r="H4" s="181" t="str">
         <f>'AVG target price'!B6</f>
@@ -13612,7 +13641,7 @@
       </c>
       <c r="I4" s="207">
         <f ca="1">'AVG target price'!C6</f>
-        <v>211.43953054210223</v>
+        <v>211.53468998587189</v>
       </c>
       <c r="K4" s="244" t="s">
         <v>436</v>
@@ -13624,7 +13653,7 @@
       </c>
       <c r="C5" s="204" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>660.81</v>
+        <v>676.76499999999999</v>
       </c>
       <c r="E5" s="181" t="s">
         <v>242</v>
@@ -13639,7 +13668,7 @@
       </c>
       <c r="I5" s="207">
         <f ca="1">'AVG target price'!C7</f>
-        <v>145.83400832217521</v>
+        <v>145.94426947147235</v>
       </c>
       <c r="K5" s="244" t="s">
         <v>437</v>
@@ -13649,16 +13678,16 @@
       <c r="B6" s="181" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="204" cm="1">
-        <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>660.9</v>
+      <c r="C6" s="204" t="e" cm="1" vm="2">
+        <f t="array" ref="C6">_FV(C3,"Price (Extended hours)",TRUE)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E6" s="181" t="s">
         <v>236</v>
       </c>
       <c r="F6" s="186">
         <f ca="1">Statement!AC148</f>
-        <v>47.608789625360224</v>
+        <v>48.758285302593656</v>
       </c>
       <c r="H6" s="181" t="str">
         <f>'AVG target price'!B8</f>
@@ -13666,7 +13695,7 @@
       </c>
       <c r="I6" s="207">
         <f ca="1">'AVG target price'!C8</f>
-        <v>226.51749630369039</v>
+        <v>226.62043250032397</v>
       </c>
       <c r="K6" s="245" t="s">
         <v>438</v>
@@ -13678,14 +13707,14 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>21.8</v>
+        <v>15.955</v>
       </c>
       <c r="E7" s="182" t="s">
         <v>200</v>
       </c>
       <c r="F7" s="187">
         <f ca="1">Statement!AC149</f>
-        <v>12.395267527675276</v>
+        <v>12.69454643296433</v>
       </c>
       <c r="H7" s="181" t="str">
         <f>'AVG target price'!B9</f>
@@ -13693,23 +13722,23 @@
       </c>
       <c r="I7" s="207">
         <f ca="1">'AVG target price'!C9</f>
-        <v>217.72301241502359</v>
+        <v>217.82141268626447</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B8" s="181" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="6" cm="1">
-        <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>0.09</v>
+      <c r="C8" s="6" t="e" cm="1" vm="3">
+        <f t="array" ref="C8">_FV(C3,"Change (extended hours)",TRUE)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E8" s="181" t="s">
         <v>264</v>
       </c>
       <c r="F8" s="188">
         <f ca="1">Statement!AC159</f>
-        <v>1.8466021466941512E-2</v>
+        <v>1.8030677776731393E-2</v>
       </c>
       <c r="H8" s="180" t="str">
         <f>'AVG target price'!B10</f>
@@ -13717,7 +13746,7 @@
       </c>
       <c r="I8" s="208">
         <f ca="1">'AVG target price'!C10</f>
-        <v>186.97493680350297</v>
+        <v>187.07893416333746</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.2">
@@ -13726,14 +13755,14 @@
       </c>
       <c r="C9" s="73" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>3.4114999999999999E-2</v>
+        <v>2.4145E-2</v>
       </c>
       <c r="E9" s="181" t="s">
         <v>287</v>
       </c>
       <c r="F9" s="188">
         <f ca="1">Statement!AC160</f>
-        <v>2.100452474992812E-2</v>
+        <v>2.050933485035426E-2</v>
       </c>
       <c r="H9" s="180" t="str">
         <f>'AVG target price'!B12</f>
@@ -13741,23 +13770,23 @@
       </c>
       <c r="I9" s="209">
         <f ca="1">'AVG target price'!C12</f>
-        <v>-0.71705189569845651</v>
+        <v>-0.72356883975480779</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B10" s="181" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="73" cm="1">
-        <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>1.362E-4</v>
+      <c r="C10" s="73" t="e" cm="1" vm="4">
+        <f t="array" ref="C10">_FV(C3,"Change % (extended hours)",TRUE)</f>
+        <v>#VALUE!</v>
       </c>
       <c r="E10" s="181" t="s">
         <v>292</v>
       </c>
       <c r="F10" s="188">
         <f ca="1">Statement!AC162</f>
-        <v>1.1237966037972705E-3</v>
+        <v>1.0973026586115924E-3</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.2">
@@ -13773,14 +13802,14 @@
       </c>
       <c r="F11" s="189">
         <f ca="1">Statement!AC161</f>
-        <v>4.4188193277946769E-3</v>
+        <v>4.3146439310543542E-3</v>
       </c>
       <c r="H11" s="180" t="s">
         <v>362</v>
       </c>
       <c r="I11" s="208">
         <f ca="1">DDM!C26</f>
-        <v>23.515889801519197</v>
+        <v>23.547833984482043</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.2">
@@ -13805,7 +13834,7 @@
       </c>
       <c r="C13" s="205" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>2.1537000000000002</v>
+        <v>2.1414</v>
       </c>
       <c r="E13" s="181" t="s">
         <v>103</v>
@@ -13828,7 +13857,7 @@
       </c>
       <c r="C14" s="206" cm="1">
         <f t="array" aca="1" ref="C14" ca="1">_FV(C3,"Volume average",TRUE)</f>
-        <v>4841848</v>
+        <v>4841084</v>
       </c>
       <c r="E14" s="182" t="s">
         <v>104</v>
@@ -13844,7 +13873,7 @@
       </c>
       <c r="F15" s="188">
         <f ca="1">Statement!AC174</f>
-        <v>-1.1882872043560911E-2</v>
+        <v>-1.1602728679978257E-2</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.2">
@@ -13877,7 +13906,7 @@
       </c>
       <c r="I17" s="242">
         <f ca="1">DCF!C15</f>
-        <v>0.14565978630451679</v>
+        <v>0.14554164361796129</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.2">
@@ -13899,7 +13928,7 @@
       </c>
       <c r="I18" s="243">
         <f ca="1">Multiples!C54</f>
-        <v>0.14789649999999999</v>
+        <v>0.14772299999999999</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
@@ -13966,12 +13995,12 @@
       <c r="C26" s="166">
         <v>0.21</v>
       </c>
-      <c r="E26" s="181" t="e" vm="2">
+      <c r="E26" s="181" t="e" vm="5">
         <v>#VALUE!</v>
       </c>
       <c r="F26" s="215" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>50.98</v>
+        <v>51.36</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -13986,7 +14015,7 @@
       </c>
       <c r="F27" s="216">
         <f ca="1">F26/1000</f>
-        <v>5.0979999999999998E-2</v>
+        <v>5.1360000000000003E-2</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
@@ -18384,6 +18413,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -18391,12 +18426,6 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -19457,16 +19486,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="AA2:AC2"/>
+    <mergeCell ref="C4:L4"/>
+    <mergeCell ref="S4:AC4"/>
+    <mergeCell ref="C13:L13"/>
+    <mergeCell ref="C18:L18"/>
     <mergeCell ref="C31:L31"/>
     <mergeCell ref="C25:L25"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="S2:Z2"/>
-    <mergeCell ref="AA2:AC2"/>
-    <mergeCell ref="C4:L4"/>
-    <mergeCell ref="S4:AC4"/>
-    <mergeCell ref="C13:L13"/>
-    <mergeCell ref="C18:L18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -19589,7 +19618,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Overview!C5</f>
-        <v>660.81</v>
+        <v>676.76499999999999</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -19598,7 +19627,7 @@
       </c>
       <c r="C7" s="134">
         <f ca="1">C5*C6</f>
-        <v>156611.97</v>
+        <v>160393.30499999999</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -19616,7 +19645,7 @@
       </c>
       <c r="C9" s="135">
         <f ca="1">Overview!F27</f>
-        <v>5.0979999999999998E-2</v>
+        <v>5.1360000000000003E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -19625,7 +19654,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C13</f>
-        <v>2.1537000000000002</v>
+        <v>2.1414</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -19668,7 +19697,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>2.2256632773113388E-2</v>
+        <v>2.1743332855264638E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -19677,7 +19706,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.97774336722688659</v>
+        <v>0.97825666714473536</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -19695,7 +19724,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>0.14789649999999999</v>
+        <v>0.14772299999999999</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -19704,7 +19733,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>0.14565978630451679</v>
+        <v>0.14554164361796129</v>
       </c>
     </row>
   </sheetData>
@@ -19956,7 +19985,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>30138.305404321778</v>
+        <v>30165.581147678571</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -20010,23 +20039,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>3781.5443008184361</v>
+        <v>3781.9343013090484</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>4626.1027856074834</v>
+        <v>4627.057038815954</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>4395.5135513701534</v>
+        <v>4396.8736538361281</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>3428.5632075058943</v>
+        <v>3429.9778128577291</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>1965.6961389336327</v>
+        <v>1966.7099847878962</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -20045,7 +20074,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>15270.050850746456</v>
+        <v>15291.753491336116</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
@@ -20068,7 +20097,7 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.14565978630451679</v>
+        <v>0.14554164361796129</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -20083,7 +20112,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>18197.419984235599</v>
+        <v>18202.552791606755</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -20092,7 +20121,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>15270.050850746456</v>
+        <v>15291.753491336116</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -20101,7 +20130,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>33467.470834982058</v>
+        <v>33494.306282942867</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -20128,7 +20157,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>31606.470834982058</v>
+        <v>31633.306282942867</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -20146,7 +20175,7 @@
       </c>
       <c r="C26" s="241">
         <f ca="1">C24/C25</f>
-        <v>133.36063643452346</v>
+        <v>133.47386617275473</v>
       </c>
     </row>
   </sheetData>
@@ -20416,23 +20445,23 @@
       <c r="G9" s="138"/>
       <c r="H9" s="92">
         <f ca="1">DCF!H10</f>
-        <v>3781.5443008184361</v>
+        <v>3781.9343013090484</v>
       </c>
       <c r="I9" s="92">
         <f ca="1">DCF!I10</f>
-        <v>4626.1027856074834</v>
+        <v>4627.057038815954</v>
       </c>
       <c r="J9" s="92">
         <f ca="1">DCF!J10</f>
-        <v>4395.5135513701534</v>
+        <v>4396.8736538361281</v>
       </c>
       <c r="K9" s="92">
         <f ca="1">DCF!K10</f>
-        <v>3428.5632075058943</v>
+        <v>3429.9778128577291</v>
       </c>
       <c r="L9" s="92">
         <f ca="1">DCF!L10</f>
-        <v>1965.6961389336327</v>
+        <v>1966.7099847878962</v>
       </c>
       <c r="N9" s="91"/>
     </row>
@@ -21218,7 +21247,7 @@
       </c>
       <c r="C41" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.14565978630451679</v>
+        <v>0.14554164361796129</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.2">
@@ -21244,7 +21273,7 @@
       </c>
       <c r="C44" s="24">
         <f ca="1">C43/(1+C41)^5</f>
-        <v>35740.44489317626</v>
+        <v>35758.878719832777</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.2">
@@ -21253,7 +21282,7 @@
       </c>
       <c r="C45" s="108">
         <f ca="1">SUM(H9:K9)+C44</f>
-        <v>51972.168738478227</v>
+        <v>51994.721526651636</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -21280,7 +21309,7 @@
       </c>
       <c r="C48" s="108">
         <f ca="1">C45+C46-C47</f>
-        <v>50111.168738478227</v>
+        <v>50133.721526651636</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -21298,7 +21327,7 @@
       </c>
       <c r="C50" s="241">
         <f ca="1">C48/C49</f>
-        <v>211.43953054210223</v>
+        <v>211.53468998587189</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
@@ -21322,7 +21351,7 @@
       </c>
       <c r="C54" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.14789649999999999</v>
+        <v>0.14772299999999999</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.2">
@@ -21357,7 +21386,7 @@
       </c>
       <c r="C58" s="241">
         <f ca="1">C57/(1+C54)^5</f>
-        <v>145.83400832217521</v>
+        <v>145.94426947147235</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
@@ -21381,7 +21410,7 @@
       </c>
       <c r="C62" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.14565978630451679</v>
+        <v>0.14554164361796129</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
@@ -21407,7 +21436,7 @@
       </c>
       <c r="C65" s="24">
         <f ca="1">C64/(1+C62)^5</f>
-        <v>39313.922778672655</v>
+        <v>39334.199695757925</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
@@ -21416,7 +21445,7 @@
       </c>
       <c r="C66" s="108">
         <f ca="1">SUM(H9:K9)+C65</f>
-        <v>55545.646623974622</v>
+        <v>55570.042502576784</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.2">
@@ -21443,7 +21472,7 @@
       </c>
       <c r="C69" s="108">
         <f ca="1">C66+C67-C68</f>
-        <v>53684.646623974622</v>
+        <v>53709.042502576784</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.2">
@@ -21461,7 +21490,7 @@
       </c>
       <c r="C71" s="241">
         <f ca="1">C69/C70</f>
-        <v>226.51749630369039</v>
+        <v>226.62043250032397</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.2">
@@ -21485,7 +21514,7 @@
       </c>
       <c r="C75" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.14565978630451679</v>
+        <v>0.14554164361796129</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.2">
@@ -21511,7 +21540,7 @@
       </c>
       <c r="C78" s="24">
         <f ca="1">C77/(1+C75)^5</f>
-        <v>37229.630097058624</v>
+        <v>37248.831999825823</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.2">
@@ -21520,7 +21549,7 @@
       </c>
       <c r="C79" s="108">
         <f ca="1">SUM(H9:K9)+C78</f>
-        <v>53461.353942360591</v>
+        <v>53484.674806644682</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.2">
@@ -21547,7 +21576,7 @@
       </c>
       <c r="C82" s="108">
         <f ca="1">C79+C80-C81</f>
-        <v>51600.353942360591</v>
+        <v>51623.674806644682</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.2">
@@ -21565,22 +21594,22 @@
       </c>
       <c r="C84" s="241">
         <f ca="1">C82/C83</f>
-        <v>217.72301241502359</v>
+        <v>217.82141268626447</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="C27:L27"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B60:C60"/>
     <mergeCell ref="C22:L22"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="C17:L17"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="C27:L27"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B60:C60"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -21631,7 +21660,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>133.36063643452346</v>
+        <v>133.47386617275473</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -21640,7 +21669,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Multiples!C50</f>
-        <v>211.43953054210223</v>
+        <v>211.53468998587189</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -21649,7 +21678,7 @@
       </c>
       <c r="C7" s="133">
         <f ca="1">Multiples!C58</f>
-        <v>145.83400832217521</v>
+        <v>145.94426947147235</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -21658,7 +21687,7 @@
       </c>
       <c r="C8" s="133">
         <f ca="1">Multiples!C71</f>
-        <v>226.51749630369039</v>
+        <v>226.62043250032397</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -21667,7 +21696,7 @@
       </c>
       <c r="C9" s="133">
         <f ca="1">Multiples!C84</f>
-        <v>217.72301241502359</v>
+        <v>217.82141268626447</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -21676,7 +21705,7 @@
       </c>
       <c r="C10" s="241">
         <f ca="1">AVERAGE(C5:C9)</f>
-        <v>186.97493680350297</v>
+        <v>187.07893416333746</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -21685,7 +21714,7 @@
       </c>
       <c r="C11" s="133">
         <f ca="1">Overview!C5</f>
-        <v>660.81</v>
+        <v>676.76499999999999</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -21694,7 +21723,7 @@
       </c>
       <c r="C12" s="152">
         <f ca="1">(C10-C11)/C11</f>
-        <v>-0.71705189569845651</v>
+        <v>-0.72356883975480779</v>
       </c>
     </row>
   </sheetData>
@@ -22204,7 +22233,7 @@
       </c>
       <c r="C24" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.14789649999999999</v>
+        <v>0.14772299999999999</v>
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
@@ -22221,7 +22250,7 @@
       </c>
       <c r="C26" s="241">
         <f ca="1">C23/(C24-C25)</f>
-        <v>23.515889801519197</v>
+        <v>23.547833984482043</v>
       </c>
     </row>
   </sheetData>
@@ -22459,7 +22488,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>258874.2575445894</v>
+        <v>259108.54370354029</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22513,23 +22542,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>4329.1795102865008</v>
+        <v>4329.6259898193721</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>6083.8122232114756</v>
+        <v>6085.0671666493508</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>8549.6041638725874</v>
+        <v>8552.249665375537</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>12014.790837893786</v>
+        <v>12019.748071111262</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>16884.430683741743</v>
+        <v>16893.139155875997</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22548,15 +22577,15 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>131162.75197371442</v>
+        <v>131349.16772914704</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B14" s="261" t="s">
+      <c r="B14" s="262" t="s">
         <v>221</v>
       </c>
-      <c r="C14" s="262"/>
+      <c r="C14" s="263"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B15" s="153" t="s">
@@ -22564,7 +22593,7 @@
       </c>
       <c r="C15" s="154">
         <f ca="1">Overview!C5</f>
-        <v>660.81</v>
+        <v>676.76499999999999</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -22573,7 +22602,7 @@
       </c>
       <c r="C16" s="154">
         <f ca="1">C36</f>
-        <v>780.45625283136792</v>
+        <v>781.3568184051918</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -22583,20 +22612,20 @@
       <c r="C17" s="156">
         <v>0.61</v>
       </c>
-      <c r="E17" s="263" t="s">
+      <c r="E17" s="261" t="s">
         <v>224</v>
       </c>
-      <c r="F17" s="263"/>
-      <c r="G17" s="263"/>
-      <c r="H17" s="263"/>
-      <c r="I17" s="263"/>
+      <c r="F17" s="261"/>
+      <c r="G17" s="261"/>
+      <c r="H17" s="261"/>
+      <c r="I17" s="261"/>
     </row>
     <row r="18" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="261" t="s">
+      <c r="B19" s="262" t="s">
         <v>183</v>
       </c>
-      <c r="C19" s="262"/>
+      <c r="C19" s="263"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="157" t="s">
@@ -22612,7 +22641,7 @@
       </c>
       <c r="C21" s="218">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.14565978630451679</v>
+        <v>0.14554164361796129</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -22630,7 +22659,7 @@
       </c>
       <c r="C23" s="159">
         <f ca="1">C15*C22</f>
-        <v>150003.87</v>
+        <v>153625.655</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -22657,15 +22686,15 @@
       </c>
       <c r="C26" s="160">
         <f ca="1">C23+C25-C24</f>
-        <v>151864.87</v>
+        <v>155486.655</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="261" t="s">
+      <c r="B28" s="262" t="s">
         <v>185</v>
       </c>
-      <c r="C28" s="262"/>
+      <c r="C28" s="263"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="157" t="s">
@@ -22673,7 +22702,7 @@
       </c>
       <c r="C29" s="159">
         <f ca="1">SUM(H10:L10)</f>
-        <v>47861.817419006096</v>
+        <v>47879.830048831514</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -22682,7 +22711,7 @@
       </c>
       <c r="C30" s="159">
         <f ca="1">L11</f>
-        <v>131162.75197371442</v>
+        <v>131349.16772914704</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -22691,7 +22720,7 @@
       </c>
       <c r="C31" s="162">
         <f ca="1">C29+C30</f>
-        <v>179024.56939272053</v>
+        <v>179228.99777797854</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -22718,7 +22747,7 @@
       </c>
       <c r="C34" s="162">
         <f ca="1">C31+C32-C33</f>
-        <v>177163.56939272053</v>
+        <v>177367.99777797854</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
@@ -22736,21 +22765,21 @@
       </c>
       <c r="C36" s="165">
         <f ca="1">C34/C35</f>
-        <v>780.45625283136792</v>
+        <v>781.3568184051918</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
+    <mergeCell ref="B14:C14"/>
     <mergeCell ref="E17:I17"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
-    <mergeCell ref="B14:C14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -29531,7 +29560,7 @@
       </c>
       <c r="AC114" s="63">
         <f ca="1">Overview!C5</f>
-        <v>660.81</v>
+        <v>676.76499999999999</v>
       </c>
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.2">
@@ -29605,7 +29634,7 @@
       </c>
       <c r="AC115" s="65">
         <f ca="1">AC114/AC84</f>
-        <v>660.81</v>
+        <v>676.76499999999999</v>
       </c>
     </row>
     <row r="117" spans="1:31" x14ac:dyDescent="0.2">
@@ -30974,7 +31003,7 @@
       <c r="AA148" s="49"/>
       <c r="AC148" s="72">
         <f ca="1">AC115/Statement!AC25</f>
-        <v>47.608789625360224</v>
+        <v>48.758285302593656</v>
       </c>
     </row>
     <row r="149" spans="2:29" x14ac:dyDescent="0.2">
@@ -31015,7 +31044,7 @@
       <c r="AA149" s="49"/>
       <c r="AC149" s="72">
         <f ca="1">AC115/(Statement!AC5/Statement!AC21)</f>
-        <v>12.395267527675276</v>
+        <v>12.69454643296433</v>
       </c>
     </row>
     <row r="150" spans="2:29" x14ac:dyDescent="0.2">
@@ -31080,7 +31109,7 @@
       </c>
       <c r="AC150" s="72">
         <f ca="1">AC115/(Statement!AC48/Statement!AC74)</f>
-        <v>69.221905860636824</v>
+        <v>70.893241808952467</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -31145,7 +31174,7 @@
       </c>
       <c r="AC151" s="141">
         <f ca="1">Statement!AC115*Statement!AC77</f>
-        <v>156611.97</v>
+        <v>160393.30499999999</v>
       </c>
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
@@ -31210,7 +31239,7 @@
       </c>
       <c r="AC152" s="141">
         <f ca="1">AC151+AC106-AC105+AC47+AC44</f>
-        <v>158472.97</v>
+        <v>162254.30499999999</v>
       </c>
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
@@ -31251,7 +31280,7 @@
       <c r="AA153" s="49"/>
       <c r="AC153" s="179">
         <f ca="1">AC152/AC5</f>
-        <v>12.994913489134891</v>
+        <v>13.304986059860598</v>
       </c>
     </row>
     <row r="154" spans="2:29" x14ac:dyDescent="0.2">
@@ -31292,7 +31321,7 @@
       <c r="AA154" s="49"/>
       <c r="AC154" s="179">
         <f ca="1">AC152/AC11</f>
-        <v>38.708590620420125</v>
+        <v>39.632219101123596</v>
       </c>
     </row>
     <row r="155" spans="2:29" x14ac:dyDescent="0.2">
@@ -31439,7 +31468,7 @@
       <c r="AA157" s="49"/>
       <c r="AC157" s="72">
         <f t="shared" ref="AC157:AC158" ca="1" si="205">AC151/AC155</f>
-        <v>54.153516597510375</v>
+        <v>55.46103215767635</v>
       </c>
     </row>
     <row r="158" spans="2:29" x14ac:dyDescent="0.2">
@@ -31480,7 +31509,7 @@
       <c r="AA158" s="49"/>
       <c r="AC158" s="72">
         <f t="shared" ca="1" si="205"/>
-        <v>51.442232720259383</v>
+        <v>52.669699556170023</v>
       </c>
     </row>
     <row r="159" spans="2:29" x14ac:dyDescent="0.2">
@@ -31521,7 +31550,7 @@
       <c r="AA159" s="49"/>
       <c r="AC159" s="74">
         <f t="shared" ref="AC159" ca="1" si="210">AC155/AC151</f>
-        <v>1.8466021466941512E-2</v>
+        <v>1.8030677776731393E-2</v>
       </c>
     </row>
     <row r="160" spans="2:29" x14ac:dyDescent="0.2">
@@ -31562,7 +31591,7 @@
       <c r="AA160" s="49"/>
       <c r="AC160" s="74">
         <f ca="1">AC25/AC115</f>
-        <v>2.100452474992812E-2</v>
+        <v>2.050933485035426E-2</v>
       </c>
     </row>
     <row r="161" spans="2:29" x14ac:dyDescent="0.2">
@@ -31603,7 +31632,7 @@
       <c r="AA161" s="49"/>
       <c r="AC161" s="152">
         <f ca="1">AC81/AC115</f>
-        <v>4.4188193277946769E-3</v>
+        <v>4.3146439310543542E-3</v>
       </c>
     </row>
     <row r="162" spans="2:29" x14ac:dyDescent="0.2">
@@ -31644,7 +31673,7 @@
       <c r="AA162" s="49"/>
       <c r="AC162" s="152">
         <f ca="1">-AC62/AC151</f>
-        <v>1.1237966037972705E-3</v>
+        <v>1.0973026586115924E-3</v>
       </c>
     </row>
     <row r="163" spans="2:29" x14ac:dyDescent="0.2">
@@ -31685,7 +31714,7 @@
       <c r="AA163" s="49"/>
       <c r="AC163" s="152">
         <f ca="1">-(AC62+AC63)/AC151</f>
-        <v>5.1720184606578925E-3</v>
+        <v>5.0500860992919875E-3</v>
       </c>
     </row>
     <row r="164" spans="2:29" x14ac:dyDescent="0.2">
@@ -32232,7 +32261,7 @@
       <c r="AA174" s="49"/>
       <c r="AC174" s="152">
         <f ca="1">(AC105-AC106)/AC151</f>
-        <v>-1.1882872043560911E-2</v>
+        <v>-1.1602728679978257E-2</v>
       </c>
     </row>
     <row r="175" spans="2:29" x14ac:dyDescent="0.2">
@@ -33607,7 +33636,7 @@
       </c>
       <c r="C5" s="168">
         <f ca="1">Overview!C5</f>
-        <v>660.81</v>
+        <v>676.76499999999999</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="132" t="s">
@@ -33623,7 +33652,7 @@
       </c>
       <c r="C6" s="169">
         <f ca="1">Statement!AC151</f>
-        <v>156611.97</v>
+        <v>160393.30499999999</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -33643,7 +33672,7 @@
       </c>
       <c r="C7" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>158472.97</v>
+        <v>162254.30499999999</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>30</v>
@@ -33663,7 +33692,7 @@
       </c>
       <c r="C8" s="170">
         <f ca="1">Statement!AC148</f>
-        <v>47.608789625360224</v>
+        <v>48.758285302593656</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>242</v>
@@ -33683,7 +33712,7 @@
       </c>
       <c r="C9" s="170">
         <f ca="1">Statement!AC149</f>
-        <v>12.395267527675276</v>
+        <v>12.69454643296433</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>243</v>
@@ -33703,7 +33732,7 @@
       </c>
       <c r="C10" s="170">
         <f ca="1">Statement!AC150</f>
-        <v>69.221905860636824</v>
+        <v>70.893241808952467</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -33723,7 +33752,7 @@
       </c>
       <c r="C11" s="170">
         <f ca="1">Statement!AC153</f>
-        <v>12.994913489134891</v>
+        <v>13.304986059860598</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -33732,7 +33761,7 @@
       </c>
       <c r="C12" s="170">
         <f ca="1">Statement!AC154</f>
-        <v>38.708590620420125</v>
+        <v>39.632219101123596</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
@@ -33968,7 +33997,7 @@
       </c>
       <c r="C38" s="171">
         <f ca="1">Statement!AC160</f>
-        <v>2.100452474992812E-2</v>
+        <v>2.050933485035426E-2</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>269</v>
@@ -33984,7 +34013,7 @@
       </c>
       <c r="C39" s="211">
         <f ca="1">Statement!AC159</f>
-        <v>1.8466021466941512E-2</v>
+        <v>1.8030677776731393E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>271</v>
@@ -34000,7 +34029,7 @@
       </c>
       <c r="C40" s="171">
         <f ca="1">Statement!AC161</f>
-        <v>4.4188193277946769E-3</v>
+        <v>4.3146439310543542E-3</v>
       </c>
       <c r="E40" s="20" t="s">
         <v>272</v>
@@ -34016,7 +34045,7 @@
       </c>
       <c r="C41" s="171">
         <f ca="1">Statement!AC162</f>
-        <v>1.1237966037972705E-3</v>
+        <v>1.0973026586115924E-3</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
@@ -34025,7 +34054,7 @@
       </c>
       <c r="C42" s="171">
         <f ca="1">Statement!AC163</f>
-        <v>5.1720184606578925E-3</v>
+        <v>5.0500860992919875E-3</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
@@ -34069,7 +34098,7 @@
       </c>
       <c r="F48" s="171">
         <f ca="1">Statement!AC174</f>
-        <v>-1.1882872043560911E-2</v>
+        <v>-1.1602728679978257E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
@@ -34249,7 +34278,7 @@
       </c>
       <c r="I6" s="168">
         <f ca="1">Statement!AC114</f>
-        <v>660.81</v>
+        <v>676.76499999999999</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -34278,7 +34307,7 @@
       </c>
       <c r="I7" s="169">
         <f ca="1">Statement!AC151</f>
-        <v>156611.97</v>
+        <v>160393.30499999999</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -34307,7 +34336,7 @@
       </c>
       <c r="I8" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>158472.97</v>
+        <v>162254.30499999999</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -34336,7 +34365,7 @@
       </c>
       <c r="I9" s="170">
         <f ca="1">Statement!AC148</f>
-        <v>47.608789625360224</v>
+        <v>48.758285302593656</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -34365,7 +34394,7 @@
       </c>
       <c r="I10" s="170">
         <f ca="1">Statement!AC149</f>
-        <v>12.395267527675276</v>
+        <v>12.69454643296433</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -34394,7 +34423,7 @@
       </c>
       <c r="I11" s="170">
         <f ca="1">Statement!AC150</f>
-        <v>69.221905860636824</v>
+        <v>70.893241808952467</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -34423,7 +34452,7 @@
       </c>
       <c r="I12" s="170">
         <f ca="1">Statement!AC153</f>
-        <v>12.994913489134891</v>
+        <v>13.304986059860598</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -34452,7 +34481,7 @@
       </c>
       <c r="I13" s="170">
         <f ca="1">Statement!AC154</f>
-        <v>38.708590620420125</v>
+        <v>39.632219101123596</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -35225,7 +35254,7 @@
       </c>
       <c r="I51" s="171">
         <f ca="1">Statement!AC160</f>
-        <v>2.100452474992812E-2</v>
+        <v>2.050933485035426E-2</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -35254,7 +35283,7 @@
       </c>
       <c r="I52" s="171">
         <f ca="1">Statement!AC159</f>
-        <v>1.8466021466941512E-2</v>
+        <v>1.8030677776731393E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -35283,7 +35312,7 @@
       </c>
       <c r="I53" s="171">
         <f ca="1">Statement!AC161</f>
-        <v>4.4188193277946769E-3</v>
+        <v>4.3146439310543542E-3</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
@@ -35312,7 +35341,7 @@
       </c>
       <c r="I54" s="171">
         <f ca="1">Statement!AC162</f>
-        <v>1.1237966037972705E-3</v>
+        <v>1.0973026586115924E-3</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
@@ -35341,7 +35370,7 @@
       </c>
       <c r="I55" s="171">
         <f ca="1">Statement!AC163</f>
-        <v>5.1720184606578925E-3</v>
+        <v>5.0500860992919875E-3</v>
       </c>
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -35577,7 +35606,7 @@
       </c>
       <c r="I68" s="192">
         <f ca="1">Statement!AC174</f>
-        <v>-1.1882872043560911E-2</v>
+        <v>-1.1602728679978257E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -36040,14 +36069,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="250" t="s">
+      <c r="C3" s="252" t="s">
         <v>312</v>
       </c>
-      <c r="D3" s="251"/>
-      <c r="F3" s="252" t="s">
+      <c r="D3" s="253"/>
+      <c r="F3" s="254" t="s">
         <v>313</v>
       </c>
-      <c r="G3" s="251"/>
+      <c r="G3" s="253"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -36114,19 +36143,19 @@
       <c r="B7" s="202" t="s">
         <v>314</v>
       </c>
-      <c r="C7" s="253">
+      <c r="C7" s="250">
         <f>Statement!AA88</f>
         <v>0.16613110539845757</v>
       </c>
-      <c r="D7" s="254"/>
-      <c r="F7" s="253">
+      <c r="D7" s="251"/>
+      <c r="F7" s="250">
         <f>IF(F6=0,
 IF(G6=0,0,IF(G6&gt;0,1,-1)),
 (G6-F6)/ABS(F6)
 )</f>
         <v>0.484860883797054</v>
       </c>
-      <c r="G7" s="254"/>
+      <c r="G7" s="251"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="203" t="s">
@@ -36153,19 +36182,19 @@
       <c r="B9" s="202" t="s">
         <v>314</v>
       </c>
-      <c r="C9" s="253">
+      <c r="C9" s="250">
         <f>Statement!AA89</f>
         <v>3.9639639639639637E-2</v>
       </c>
-      <c r="D9" s="254"/>
-      <c r="F9" s="253">
+      <c r="D9" s="251"/>
+      <c r="F9" s="250">
         <f>IF(F8=0,
 IF(G8=0,0,IF(G8&gt;0,1,-1)),
 (G8-F8)/ABS(F8)
 )</f>
         <v>0.13137254901960785</v>
       </c>
-      <c r="G9" s="254"/>
+      <c r="G9" s="251"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="203" t="s">
@@ -36192,19 +36221,19 @@
       <c r="B11" s="202" t="s">
         <v>314</v>
       </c>
-      <c r="C11" s="253">
+      <c r="C11" s="250">
         <f>Statement!AA90</f>
         <v>0.31167933655839669</v>
       </c>
-      <c r="D11" s="254"/>
-      <c r="F11" s="253">
+      <c r="D11" s="251"/>
+      <c r="F11" s="250">
         <f>IF(F10=0,
 IF(G10=0,0,IF(G10&gt;0,1,-1)),
 (G10-F10)/ABS(F10)
 )</f>
         <v>1.0765864332603938</v>
       </c>
-      <c r="G11" s="254"/>
+      <c r="G11" s="251"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="203" t="s">
@@ -36231,19 +36260,19 @@
       <c r="B13" s="202" t="s">
         <v>314</v>
       </c>
-      <c r="C13" s="253">
+      <c r="C13" s="250">
         <f>Statement!AA93</f>
         <v>-0.24498886414253898</v>
       </c>
-      <c r="D13" s="254"/>
-      <c r="F13" s="253">
+      <c r="D13" s="251"/>
+      <c r="F13" s="250">
         <f>IF(F12=0,
 IF(G12=0,0,IF(G12&gt;0,1,-1)),
 (G12-F12)/ABS(F12)
 )</f>
         <v>-2.023121387283237E-2</v>
       </c>
-      <c r="G13" s="254"/>
+      <c r="G13" s="251"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="203" t="s">
@@ -36270,19 +36299,19 @@
       <c r="B15" s="202" t="s">
         <v>314</v>
       </c>
-      <c r="C15" s="253">
+      <c r="C15" s="250">
         <f>Statement!AA94</f>
         <v>0.56212424849699394</v>
       </c>
-      <c r="D15" s="254"/>
-      <c r="F15" s="253">
+      <c r="D15" s="251"/>
+      <c r="F15" s="250">
         <f>IF(F14=0,
 IF(G14=0,0,IF(G14&gt;0,1,-1)),
 (G14-F14)/ABS(F14)
 )</f>
         <v>1.744718309859155</v>
       </c>
-      <c r="G15" s="254"/>
+      <c r="G15" s="251"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="203" t="s">
@@ -36309,19 +36338,19 @@
       <c r="B17" s="202" t="s">
         <v>314</v>
       </c>
-      <c r="C17" s="253">
+      <c r="C17" s="250">
         <f>Statement!AA96</f>
         <v>0.72994652406417115</v>
       </c>
-      <c r="D17" s="254"/>
-      <c r="F17" s="253">
+      <c r="D17" s="251"/>
+      <c r="F17" s="250">
         <f>IF(F16=0,
 IF(G16=0,0,IF(G16&gt;0,1,-1)),
 (G16-F16)/ABS(F16)
 )</f>
         <v>1.651639344262295</v>
       </c>
-      <c r="G17" s="254"/>
+      <c r="G17" s="251"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="203" t="s">
@@ -36348,22 +36377,22 @@
       <c r="B19" s="202" t="s">
         <v>314</v>
       </c>
-      <c r="C19" s="253">
+      <c r="C19" s="250">
         <f>IF(C18=0,
 IF(D18=0,0,IF(D18&gt;0,1,-1)),
 (D18-C18)/ABS(C18)
 )</f>
         <v>1.3100436681222707E-2</v>
       </c>
-      <c r="D19" s="254"/>
-      <c r="F19" s="253">
+      <c r="D19" s="251"/>
+      <c r="F19" s="250">
         <f>IF(F18=0,
 IF(G18=0,0,IF(G18&gt;0,1,-1)),
 (G18-F18)/ABS(F18)
 )</f>
         <v>6.4220183486238536E-2</v>
       </c>
-      <c r="G19" s="254"/>
+      <c r="G19" s="251"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="203" t="s">
@@ -36390,22 +36419,22 @@
       <c r="B21" s="202" t="s">
         <v>314</v>
       </c>
-      <c r="C21" s="253">
+      <c r="C21" s="250">
         <f>IF(C20=0,
 IF(D20=0,0,IF(D20&gt;0,1,-1)),
 (D20-C20)/ABS(C20)
 )</f>
         <v>0.70642201834862384</v>
       </c>
-      <c r="D21" s="254"/>
-      <c r="F21" s="253">
+      <c r="D21" s="251"/>
+      <c r="F21" s="250">
         <f>IF(F20=0,
 IF(G20=0,0,IF(G20&gt;0,1,-1)),
 (G20-F20)/ABS(F20)
 )</f>
         <v>1.4910714285714284</v>
       </c>
-      <c r="G21" s="254"/>
+      <c r="G21" s="251"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
@@ -36454,22 +36483,22 @@
       <c r="B25" s="202" t="s">
         <v>314</v>
       </c>
-      <c r="C25" s="253">
+      <c r="C25" s="250">
         <f>IF(C24=0,
 IF(D24=0,0,IF(D24&gt;0,1,-1)),
 (D24-C24)/ABS(C24)
 )</f>
         <v>0.17319999999999999</v>
       </c>
-      <c r="D25" s="254"/>
-      <c r="F25" s="253">
+      <c r="D25" s="251"/>
+      <c r="F25" s="250">
         <f>IF(F24=0,
 IF(G24=0,0,IF(G24&gt;0,1,-1)),
 (G24-F24)/ABS(F24)
 )</f>
         <v>0.57434245840042941</v>
       </c>
-      <c r="G25" s="254"/>
+      <c r="G25" s="251"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="str">
@@ -36497,25 +36526,37 @@
       <c r="B27" s="202" t="s">
         <v>314</v>
       </c>
-      <c r="C27" s="253">
+      <c r="C27" s="250">
         <f>IF(C26=0,
 IF(D26=0,0,IF(D26&gt;0,1,-1)),
 (D26-C26)/ABS(C26)
 )</f>
         <v>0.1388888888888889</v>
       </c>
-      <c r="D27" s="254"/>
-      <c r="F27" s="253">
+      <c r="D27" s="251"/>
+      <c r="F27" s="250">
         <f>IF(F26=0,
 IF(G26=0,0,IF(G26&gt;0,1,-1)),
 (G26-F26)/ABS(F26)
 )</f>
         <v>0.19965576592082615</v>
       </c>
-      <c r="G27" s="254"/>
+      <c r="G27" s="251"/>
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
     <mergeCell ref="C25:D25"/>
     <mergeCell ref="F25:G25"/>
     <mergeCell ref="C27:D27"/>
@@ -36526,18 +36567,6 @@
     <mergeCell ref="C19:D19"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="F21:G21"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Updated WDC and STX
</commit_message>
<xml_diff>
--- a/STX.xlsx
+++ b/STX.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83C6605B-D3A9-EE4F-96F1-7D28F175514F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{635D4911-B368-C542-91F0-7A0457F3C9EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
@@ -12686,11 +12686,11 @@
     <v>Powered by Refinitiv</v>
     <v>1145</v>
     <v>217.67</v>
-    <v>2.1520000000000001</v>
+    <v>2.1669999999999998</v>
     <v>-11.65</v>
     <v>-1.8142000000000002E-2</v>
-    <v>-0.4</v>
-    <v>-6.3439999999999992E-4</v>
+    <v>0.51</v>
+    <v>8.0889999999999998E-4</v>
     <v>USD</v>
     <v>Seagate Technology Holdings plc provides mass-data storage infrastructure solution. The Company’s principal products are hard disk drives, commonly referred to as disk drives, hard drives (HDDs). In addition to HDDs, the Company produces a range of data storage products, including solid state drives (SSDs), solid state hybrid drives, storage subsystems, as well as a scalable edge-to-cloud mass data platform. Its HDD products are designed for mass capacity storage and legacy markets. Mass capacity storage involves use cases, such as hyperscale data centers and public clouds, as well as emerging use cases. The Company’s HDD and SSD product portfolio includes Serial Advanced Technology Attachment, Serial Attached SCSI and Non-Volatile Memory Express based designs to support a variety of mass capacity and legacy applications. Its systems portfolio includes storage subsystems for enterprises, cloud service providers, scale-out storage servers and original equipment manufacturers.</v>
     <v>30000</v>
@@ -12701,21 +12701,20 @@
     <v>655.6</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46318.953264421092</v>
+    <v>46318.999900555471</v>
     <v>0</v>
     <v>621.00009999999997</v>
-    <v>144407997041</v>
     <v>SEAGATE TECHNOLOGY HOLDINGS PUBLIC LIMITED COMPANY</v>
     <v>SEAGATE TECHNOLOGY HOLDINGS PUBLIC LIMITED COMPANY</v>
     <v>633</v>
-    <v>45.346299999999999</v>
+    <v>46.184100000000001</v>
     <v>642.14</v>
     <v>630.49</v>
-    <v>630.09</v>
+    <v>631</v>
     <v>229040900</v>
     <v>STX</v>
     <v>SEAGATE TECHNOLOGY HOLDINGS PUBLIC LIMITED COMPANY (XNAS:STX)</v>
-    <v>5569310</v>
+    <v>5572336</v>
     <v>4901617</v>
     <v>2017</v>
   </rv>
@@ -12740,17 +12739,17 @@
     <v>Powered by Refinitiv</v>
     <v>53.64</v>
     <v>39.47</v>
-    <v>-1.93</v>
-    <v>-3.7505000000000004E-2</v>
+    <v>0.35</v>
+    <v>7.0660000000000002E-3</v>
     <v>US</v>
-    <v>50.54</v>
+    <v>50.03</v>
     <v>Index</v>
     <v>3</v>
-    <v>49.39</v>
+    <v>49.55</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>50.4</v>
-    <v>51.46</v>
+    <v>49.92</v>
     <v>49.53</v>
+    <v>49.88</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
@@ -12798,7 +12797,6 @@
     <k n="Last trade time"/>
     <k n="LearnMoreOnLink" t="r"/>
     <k n="Low"/>
-    <k n="Market cap"/>
     <k n="Name" t="s"/>
     <k n="Official name" t="s"/>
     <k n="Open"/>
@@ -12850,7 +12848,7 @@
 <file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
 <supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
   <spbArrays count="2">
-    <a count="45">
+    <a count="44">
       <v t="s">%EntityServiceId</v>
       <v t="s">_Format</v>
       <v t="s">%IsRefreshable</v>
@@ -12880,7 +12878,6 @@
       <v t="s">52 week low</v>
       <v t="s">Volume</v>
       <v t="s">Volume average</v>
-      <v t="s">Market cap</v>
       <v t="s">Beta</v>
       <v t="s">P/E</v>
       <v t="s">Shares outstanding</v>
@@ -12955,14 +12952,13 @@
       <v>4</v>
       <v>4</v>
       <v>5</v>
-      <v>6</v>
       <v>1</v>
       <v>1</v>
       <v>1</v>
       <v>4</v>
+      <v>6</v>
       <v>7</v>
       <v>8</v>
-      <v>9</v>
       <v>4</v>
       <v>1</v>
       <v>1</v>
@@ -12972,9 +12968,9 @@
       <v>at close</v>
       <v>from previous close</v>
       <v>from previous close</v>
-      <v>Source: Nasdaq Last Sale</v>
+      <v>Source: Nasdaq</v>
       <v>GMT</v>
-      <v>Real-Time Nasdaq Last Sale</v>
+      <v>Delayed 15 minutes</v>
       <v>from close</v>
       <v>from close</v>
     </spb>
@@ -12999,7 +12995,7 @@
       <v>1</v>
       <v>1</v>
       <v>1</v>
-      <v>9</v>
+      <v>8</v>
     </spb>
     <spb s="7">
       <v>from previous close</v>
@@ -13039,7 +13035,6 @@
     <k n="Volume" t="i"/>
     <k n="Employees" t="i"/>
     <k n="Change (%)" t="i"/>
-    <k n="Market cap" t="i"/>
     <k n="52 week low" t="i"/>
     <k n="52 week high" t="i"/>
     <k n="Previous close" t="i"/>
@@ -13130,9 +13125,6 @@
       <rpv i="0">#,##0</rpv>
     </rSty>
     <rSty dxfid="3"/>
-    <rSty dxfid="1">
-      <rpv i="0">_([$$-en-US]* #,##0_);_([$$-en-US]* (#,##0);_([$$-en-US]* "-"_);_(@_)</rpv>
-    </rSty>
     <rSty dxfid="2"/>
     <rSty dxfid="6">
       <rpv i="0">0</rpv>
@@ -13591,7 +13583,7 @@
       </c>
       <c r="I3" s="207">
         <f ca="1">'AVG target price'!C5</f>
-        <v>134.90700212028807</v>
+        <v>133.9327675614613</v>
       </c>
       <c r="K3" s="244" t="s">
         <v>435</v>
@@ -13618,7 +13610,7 @@
       </c>
       <c r="I4" s="207">
         <f ca="1">'AVG target price'!C6</f>
-        <v>212.7297108409131</v>
+        <v>211.91923684881951</v>
       </c>
       <c r="K4" s="244" t="s">
         <v>436</v>
@@ -13645,7 +13637,7 @@
       </c>
       <c r="I5" s="207">
         <f ca="1">'AVG target price'!C7</f>
-        <v>146.80755643991765</v>
+        <v>146.15299051680003</v>
       </c>
       <c r="K5" s="244" t="s">
         <v>437</v>
@@ -13657,7 +13649,7 @@
       </c>
       <c r="C6" s="204" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>630.09</v>
+        <v>631</v>
       </c>
       <c r="E6" s="181" t="s">
         <v>236</v>
@@ -13672,7 +13664,7 @@
       </c>
       <c r="I6" s="207">
         <f ca="1">'AVG target price'!C8</f>
-        <v>227.91314035012334</v>
+        <v>227.03640893522405</v>
       </c>
       <c r="K6" s="245" t="s">
         <v>438</v>
@@ -13699,7 +13691,7 @@
       </c>
       <c r="I7" s="207">
         <f ca="1">'AVG target price'!C9</f>
-        <v>219.05714290956459</v>
+        <v>218.21905728061432</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.2">
@@ -13708,7 +13700,7 @@
       </c>
       <c r="C8" s="6" cm="1">
         <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>-0.4</v>
+        <v>0.51</v>
       </c>
       <c r="E8" s="181" t="s">
         <v>264</v>
@@ -13723,7 +13715,7 @@
       </c>
       <c r="I8" s="208">
         <f ca="1">'AVG target price'!C10</f>
-        <v>188.28291053216134</v>
+        <v>187.45209222858384</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.2">
@@ -13747,7 +13739,7 @@
       </c>
       <c r="I9" s="209">
         <f ca="1">'AVG target price'!C12</f>
-        <v>-0.70137050463582085</v>
+        <v>-0.70268823894338706</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.2">
@@ -13756,7 +13748,7 @@
       </c>
       <c r="C10" s="73" cm="1">
         <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>-6.3439999999999992E-4</v>
+        <v>8.0889999999999998E-4</v>
       </c>
       <c r="E10" s="181" t="s">
         <v>292</v>
@@ -13786,7 +13778,7 @@
       </c>
       <c r="I11" s="208">
         <f ca="1">DDM!C26</f>
-        <v>23.799952520376671</v>
+        <v>23.608461870560067</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.2">
@@ -13811,7 +13803,7 @@
       </c>
       <c r="C13" s="205" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>2.1520000000000001</v>
+        <v>2.1669999999999998</v>
       </c>
       <c r="E13" s="181" t="s">
         <v>103</v>
@@ -13848,7 +13840,7 @@
       </c>
       <c r="I14" s="247">
         <f ca="1">'Reverse DCF'!C16</f>
-        <v>683.91677475151334</v>
+        <v>677.27257217592853</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.2">
@@ -13890,7 +13882,7 @@
       </c>
       <c r="I17" s="242">
         <f ca="1">DCF!C15</f>
-        <v>0.14406380061445392</v>
+        <v>0.14506491605983957</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.2">
@@ -13912,7 +13904,7 @@
       </c>
       <c r="I18" s="243">
         <f ca="1">Multiples!C54</f>
-        <v>0.14637</v>
+        <v>0.147395</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
@@ -13984,7 +13976,7 @@
       </c>
       <c r="F26" s="215" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>49.53</v>
+        <v>49.88</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -13999,7 +13991,7 @@
       </c>
       <c r="F27" s="216">
         <f ca="1">F26/1000</f>
-        <v>4.9530000000000005E-2</v>
+        <v>4.9880000000000001E-2</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
@@ -19629,7 +19621,7 @@
       </c>
       <c r="C9" s="135">
         <f ca="1">Overview!F27</f>
-        <v>4.9530000000000005E-2</v>
+        <v>4.9880000000000001E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -19638,7 +19630,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C13</f>
-        <v>2.1520000000000001</v>
+        <v>2.1669999999999998</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -19708,7 +19700,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>0.14637</v>
+        <v>0.147395</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -19717,7 +19709,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>0.14406380061445392</v>
+        <v>0.14506491605983957</v>
       </c>
     </row>
   </sheetData>
@@ -19969,7 +19961,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>30510.991656540005</v>
+        <v>30276.147196352598</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -20023,23 +20015,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>3786.8196102786287</v>
+        <v>3783.5088428735944</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>4639.0187500391494</v>
+        <v>4630.910627821946</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>4413.9346417391207</v>
+        <v>4402.3676226342159</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>3447.7348607503491</v>
+        <v>3435.6934237919982</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>1979.4453200085995</v>
+        <v>1970.8074200263175</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -20058,7 +20050,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>15567.006319692429</v>
+        <v>15379.777974918255</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
@@ -20081,7 +20073,7 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.14406380061445392</v>
+        <v>0.14506491605983957</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -20096,7 +20088,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>18266.953182815847</v>
+        <v>18223.28793714807</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -20105,7 +20097,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>15567.006319692429</v>
+        <v>15379.777974918255</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -20114,7 +20106,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>33833.959502508274</v>
+        <v>33603.065912066326</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -20141,7 +20133,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>31972.959502508274</v>
+        <v>31742.065912066326</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -20159,7 +20151,7 @@
       </c>
       <c r="C26" s="241">
         <f ca="1">C24/C25</f>
-        <v>134.90700212028807</v>
+        <v>133.9327675614613</v>
       </c>
     </row>
   </sheetData>
@@ -20429,23 +20421,23 @@
       <c r="G9" s="138"/>
       <c r="H9" s="92">
         <f ca="1">DCF!H10</f>
-        <v>3786.8196102786287</v>
+        <v>3783.5088428735944</v>
       </c>
       <c r="I9" s="92">
         <f ca="1">DCF!I10</f>
-        <v>4639.0187500391494</v>
+        <v>4630.910627821946</v>
       </c>
       <c r="J9" s="92">
         <f ca="1">DCF!J10</f>
-        <v>4413.9346417391207</v>
+        <v>4402.3676226342159</v>
       </c>
       <c r="K9" s="92">
         <f ca="1">DCF!K10</f>
-        <v>3447.7348607503491</v>
+        <v>3435.6934237919982</v>
       </c>
       <c r="L9" s="92">
         <f ca="1">DCF!L10</f>
-        <v>1979.4453200085995</v>
+        <v>1970.8074200263175</v>
       </c>
       <c r="N9" s="91"/>
     </row>
@@ -21231,7 +21223,7 @@
       </c>
       <c r="C41" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.14406380061445392</v>
+        <v>0.14506491605983957</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.2">
@@ -21257,7 +21249,7 @@
       </c>
       <c r="C44" s="24">
         <f ca="1">C43/(1+C41)^5</f>
-        <v>35990.433606489161</v>
+        <v>35833.378616048474</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.2">
@@ -21266,7 +21258,7 @@
       </c>
       <c r="C45" s="108">
         <f ca="1">SUM(H9:K9)+C44</f>
-        <v>52277.941469296406</v>
+        <v>52085.859133170226</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -21293,7 +21285,7 @@
       </c>
       <c r="C48" s="108">
         <f ca="1">C45+C46-C47</f>
-        <v>50416.941469296406</v>
+        <v>50224.859133170226</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -21311,7 +21303,7 @@
       </c>
       <c r="C50" s="241">
         <f ca="1">C48/C49</f>
-        <v>212.7297108409131</v>
+        <v>211.91923684881951</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
@@ -21335,7 +21327,7 @@
       </c>
       <c r="C54" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.14637</v>
+        <v>0.147395</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.2">
@@ -21370,7 +21362,7 @@
       </c>
       <c r="C58" s="241">
         <f ca="1">C57/(1+C54)^5</f>
-        <v>146.80755643991765</v>
+        <v>146.15299051680003</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
@@ -21394,7 +21386,7 @@
       </c>
       <c r="C62" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.14406380061445392</v>
+        <v>0.14506491605983957</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
@@ -21420,7 +21412,7 @@
       </c>
       <c r="C65" s="24">
         <f ca="1">C64/(1+C62)^5</f>
-        <v>39588.906400171989</v>
+        <v>39416.148400526348</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
@@ -21429,7 +21421,7 @@
       </c>
       <c r="C66" s="108">
         <f ca="1">SUM(H9:K9)+C65</f>
-        <v>55876.414262979233</v>
+        <v>55668.6289176481</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.2">
@@ -21456,7 +21448,7 @@
       </c>
       <c r="C69" s="108">
         <f ca="1">C66+C67-C68</f>
-        <v>54015.414262979233</v>
+        <v>53807.6289176481</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.2">
@@ -21474,7 +21466,7 @@
       </c>
       <c r="C71" s="241">
         <f ca="1">C69/C70</f>
-        <v>227.91314035012334</v>
+        <v>227.03640893522405</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.2">
@@ -21498,7 +21490,7 @@
       </c>
       <c r="C75" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.14406380061445392</v>
+        <v>0.14506491605983957</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.2">
@@ -21524,7 +21516,7 @@
       </c>
       <c r="C78" s="24">
         <f ca="1">C77/(1+C75)^5</f>
-        <v>37490.035006759557</v>
+        <v>37326.436058383842</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.2">
@@ -21533,7 +21525,7 @@
       </c>
       <c r="C79" s="108">
         <f ca="1">SUM(H9:K9)+C78</f>
-        <v>53777.542869566809</v>
+        <v>53578.916575505595</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.2">
@@ -21560,7 +21552,7 @@
       </c>
       <c r="C82" s="108">
         <f ca="1">C79+C80-C81</f>
-        <v>51916.542869566809</v>
+        <v>51717.916575505595</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.2">
@@ -21578,7 +21570,7 @@
       </c>
       <c r="C84" s="241">
         <f ca="1">C82/C83</f>
-        <v>219.05714290956459</v>
+        <v>218.21905728061432</v>
       </c>
     </row>
   </sheetData>
@@ -21644,7 +21636,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>134.90700212028807</v>
+        <v>133.9327675614613</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -21653,7 +21645,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Multiples!C50</f>
-        <v>212.7297108409131</v>
+        <v>211.91923684881951</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -21662,7 +21654,7 @@
       </c>
       <c r="C7" s="133">
         <f ca="1">Multiples!C58</f>
-        <v>146.80755643991765</v>
+        <v>146.15299051680003</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -21671,7 +21663,7 @@
       </c>
       <c r="C8" s="133">
         <f ca="1">Multiples!C71</f>
-        <v>227.91314035012334</v>
+        <v>227.03640893522405</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -21680,7 +21672,7 @@
       </c>
       <c r="C9" s="133">
         <f ca="1">Multiples!C84</f>
-        <v>219.05714290956459</v>
+        <v>218.21905728061432</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -21689,7 +21681,7 @@
       </c>
       <c r="C10" s="241">
         <f ca="1">AVERAGE(C5:C9)</f>
-        <v>188.28291053216134</v>
+        <v>187.45209222858384</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -21707,7 +21699,7 @@
       </c>
       <c r="C12" s="152">
         <f ca="1">(C10-C11)/C11</f>
-        <v>-0.70137050463582085</v>
+        <v>-0.70268823894338706</v>
       </c>
     </row>
   </sheetData>
@@ -22217,7 +22209,7 @@
       </c>
       <c r="C24" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.14637</v>
+        <v>0.147395</v>
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
@@ -22234,7 +22226,7 @@
       </c>
       <c r="C26" s="241">
         <f ca="1">C23/(C24-C25)</f>
-        <v>23.799952520376671</v>
+        <v>23.608461870560067</v>
       </c>
     </row>
   </sheetData>
@@ -22472,7 +22464,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>223830.86427120928</v>
+        <v>222108.02815087669</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22526,23 +22518,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>4200.584655285299</v>
+        <v>4196.9121384532173</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>5727.7505491613565</v>
+        <v>5717.7395308868854</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>7810.1333613499082</v>
+        <v>7789.6663700745248</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>10649.5879313393</v>
+        <v>10612.393556804442</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>14521.355508291239</v>
+        <v>14457.987242838353</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22561,7 +22553,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>114200.69586316642</v>
+        <v>112827.17504487834</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
@@ -22586,7 +22578,7 @@
       </c>
       <c r="C16" s="154">
         <f ca="1">C36</f>
-        <v>683.91677475151334</v>
+        <v>677.27257217592853</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -22625,7 +22617,7 @@
       </c>
       <c r="C21" s="218">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.14406380061445392</v>
+        <v>0.14506491605983957</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -22686,7 +22678,7 @@
       </c>
       <c r="C29" s="159">
         <f ca="1">SUM(H10:L10)</f>
-        <v>42909.412005427104</v>
+        <v>42774.698839057419</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -22695,7 +22687,7 @@
       </c>
       <c r="C30" s="159">
         <f ca="1">L11</f>
-        <v>114200.69586316642</v>
+        <v>112827.17504487834</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -22704,7 +22696,7 @@
       </c>
       <c r="C31" s="162">
         <f ca="1">C29+C30</f>
-        <v>157110.10786859354</v>
+        <v>155601.87388393577</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -22731,7 +22723,7 @@
       </c>
       <c r="C34" s="162">
         <f ca="1">C31+C32-C33</f>
-        <v>155249.10786859354</v>
+        <v>153740.87388393577</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
@@ -22749,7 +22741,7 @@
       </c>
       <c r="C36" s="165">
         <f ca="1">C34/C35</f>
-        <v>683.91677475151334</v>
+        <v>677.27257217592853</v>
       </c>
     </row>
   </sheetData>

</xml_diff>